<commit_message>
BDD enrichie automatiquement - 3780 nouv. lignes
</commit_message>
<xml_diff>
--- a/data/processed/clubmed_bdd.xlsx
+++ b/data/processed/clubmed_bdd.xlsx
@@ -35769,10 +35769,8 @@
           <t>Accessoire brosse à cils</t>
         </is>
       </c>
-      <c r="D1962" t="inlineStr">
-        <is>
-          <t>392690</t>
-        </is>
+      <c r="D1962" t="n">
+        <v>392690</v>
       </c>
       <c r="E1962" t="inlineStr"/>
       <c r="F1962" t="inlineStr">
@@ -35789,10 +35787,8 @@
           <t>accessoire brosse à dent</t>
         </is>
       </c>
-      <c r="D1963" t="inlineStr">
-        <is>
-          <t>392690</t>
-        </is>
+      <c r="D1963" t="n">
+        <v>392690</v>
       </c>
       <c r="E1963" t="inlineStr"/>
       <c r="F1963" t="inlineStr">
@@ -35809,10 +35805,8 @@
           <t>Attache pour ballon géant 140 - Zibi SKU:GAATT140</t>
         </is>
       </c>
-      <c r="D1964" t="inlineStr">
-        <is>
-          <t>392690</t>
-        </is>
+      <c r="D1964" t="n">
+        <v>392690</v>
       </c>
       <c r="E1964" t="inlineStr"/>
       <c r="F1964" t="inlineStr">
@@ -35829,10 +35823,8 @@
           <t>Ballon Standard Blanc HG3' - Balloonia SKU:HG3-P20</t>
         </is>
       </c>
-      <c r="D1965" t="inlineStr">
-        <is>
-          <t>950300</t>
-        </is>
+      <c r="D1965" t="n">
+        <v>950300</v>
       </c>
       <c r="E1965" t="inlineStr"/>
       <c r="F1965" t="inlineStr">
@@ -35849,10 +35841,8 @@
           <t>Ballon Standard Gris HG3' - Balloonia SKU:HG3-P44</t>
         </is>
       </c>
-      <c r="D1966" t="inlineStr">
-        <is>
-          <t>950300</t>
-        </is>
+      <c r="D1966" t="n">
+        <v>950300</v>
       </c>
       <c r="E1966" t="inlineStr"/>
       <c r="F1966" t="inlineStr">
@@ -35869,10 +35859,8 @@
           <t>liquide à bulles de savon 5l SKU:ese64391</t>
         </is>
       </c>
-      <c r="D1967" t="inlineStr">
-        <is>
-          <t>340130</t>
-        </is>
+      <c r="D1967" t="n">
+        <v>340130</v>
       </c>
       <c r="E1967" t="inlineStr"/>
       <c r="F1967" t="inlineStr">
@@ -35889,10 +35877,8 @@
           <t>lot 150 feuilles</t>
         </is>
       </c>
-      <c r="D1968" t="inlineStr">
-        <is>
-          <t>480640</t>
-        </is>
+      <c r="D1968" t="n">
+        <v>480640</v>
       </c>
       <c r="E1968" t="inlineStr"/>
       <c r="F1968" t="inlineStr">
@@ -35909,10 +35895,8 @@
           <t>lunettes led's lumineuses futuriste cyberpunk 7 couleurs SKU:lp00965 promo</t>
         </is>
       </c>
-      <c r="D1969" t="inlineStr">
-        <is>
-          <t>900490</t>
-        </is>
+      <c r="D1969" t="n">
+        <v>900490</v>
       </c>
       <c r="E1969" t="inlineStr"/>
       <c r="F1969" t="inlineStr">
@@ -35929,10 +35913,8 @@
           <t>lunettes led's lumineuses futuriste cyberpunk 7 couleurs SKU:lp0905 promo</t>
         </is>
       </c>
-      <c r="D1970" t="inlineStr">
-        <is>
-          <t>900490</t>
-        </is>
+      <c r="D1970" t="n">
+        <v>900490</v>
       </c>
       <c r="E1970" t="inlineStr"/>
       <c r="F1970" t="inlineStr">
@@ -35949,10 +35931,8 @@
           <t>machine à bulles - bubble maker SKU:ese64417</t>
         </is>
       </c>
-      <c r="D1971" t="inlineStr">
-        <is>
-          <t>847990</t>
-        </is>
+      <c r="D1971" t="n">
+        <v>847990</v>
       </c>
       <c r="E1971" t="inlineStr"/>
       <c r="F1971" t="inlineStr">
@@ -35969,10 +35949,8 @@
           <t>masque nuit</t>
         </is>
       </c>
-      <c r="D1972" t="inlineStr">
-        <is>
-          <t>630790</t>
-        </is>
+      <c r="D1972" t="n">
+        <v>630790</v>
       </c>
       <c r="E1972" t="inlineStr"/>
       <c r="F1972" t="inlineStr">
@@ -35989,10 +35967,8 @@
           <t>plante verte artificiel dans pot</t>
         </is>
       </c>
-      <c r="D1973" t="inlineStr">
-        <is>
-          <t>670210</t>
-        </is>
+      <c r="D1973" t="n">
+        <v>670210</v>
       </c>
       <c r="E1973" t="inlineStr"/>
       <c r="F1973" t="inlineStr">
@@ -36009,10 +35985,8 @@
           <t>tuyau métal 125mm, 3m</t>
         </is>
       </c>
-      <c r="D1974" t="inlineStr">
-        <is>
-          <t>732690</t>
-        </is>
+      <c r="D1974" t="n">
+        <v>732690</v>
       </c>
       <c r="E1974" t="inlineStr"/>
       <c r="F1974" t="inlineStr">
@@ -36029,10 +36003,8 @@
           <t>Canne metallique droite or</t>
         </is>
       </c>
-      <c r="D1975" t="inlineStr">
-        <is>
-          <t>950590</t>
-        </is>
+      <c r="D1975" t="n">
+        <v>950590</v>
       </c>
       <c r="E1975" t="inlineStr"/>
       <c r="F1975" t="inlineStr">
@@ -36049,10 +36021,8 @@
           <t>Costume Arlequin femme M WITHOUT BRAND</t>
         </is>
       </c>
-      <c r="D1976" t="inlineStr">
-        <is>
-          <t>950590</t>
-        </is>
+      <c r="D1976" t="n">
+        <v>950590</v>
       </c>
       <c r="E1976" t="inlineStr"/>
       <c r="F1976" t="inlineStr">
@@ -36069,10 +36039,8 @@
           <t>Costume Arlequin Venitien homme L WITHOUT BRAND</t>
         </is>
       </c>
-      <c r="D1977" t="inlineStr">
-        <is>
-          <t>950590</t>
-        </is>
+      <c r="D1977" t="n">
+        <v>950590</v>
       </c>
       <c r="E1977" t="inlineStr"/>
       <c r="F1977" t="inlineStr">
@@ -36089,10 +36057,8 @@
           <t>Costume ballerine rouge S/M WITHOUT BRAND</t>
         </is>
       </c>
-      <c r="D1978" t="inlineStr">
-        <is>
-          <t>950590</t>
-        </is>
+      <c r="D1978" t="n">
+        <v>950590</v>
       </c>
       <c r="E1978" t="inlineStr"/>
       <c r="F1978" t="inlineStr">
@@ -36109,10 +36075,8 @@
           <t>Costume chapelier Homme  M WITHOUT BRAND</t>
         </is>
       </c>
-      <c r="D1979" t="inlineStr">
-        <is>
-          <t>950590</t>
-        </is>
+      <c r="D1979" t="n">
+        <v>950590</v>
       </c>
       <c r="E1979" t="inlineStr"/>
       <c r="F1979" t="inlineStr">
@@ -36129,10 +36093,8 @@
           <t>Costume clown coloré taille standart WITHOUT BRAND</t>
         </is>
       </c>
-      <c r="D1980" t="inlineStr">
-        <is>
-          <t>950590</t>
-        </is>
+      <c r="D1980" t="n">
+        <v>950590</v>
       </c>
       <c r="E1980" t="inlineStr"/>
       <c r="F1980" t="inlineStr">
@@ -36149,10 +36111,8 @@
           <t>Costume Clown femme L noir blanc WITHOUT BRAND</t>
         </is>
       </c>
-      <c r="D1981" t="inlineStr">
-        <is>
-          <t>950590</t>
-        </is>
+      <c r="D1981" t="n">
+        <v>950590</v>
       </c>
       <c r="E1981" t="inlineStr"/>
       <c r="F1981" t="inlineStr">
@@ -36169,10 +36129,8 @@
           <t>Costume Clown Premium M WITHOUT BRAND</t>
         </is>
       </c>
-      <c r="D1982" t="inlineStr">
-        <is>
-          <t>950590</t>
-        </is>
+      <c r="D1982" t="n">
+        <v>950590</v>
       </c>
       <c r="E1982" t="inlineStr"/>
       <c r="F1982" t="inlineStr">
@@ -36189,10 +36147,8 @@
           <t>Costume coloré femme M WITHOUT BRAND</t>
         </is>
       </c>
-      <c r="D1983" t="inlineStr">
-        <is>
-          <t>950590</t>
-        </is>
+      <c r="D1983" t="n">
+        <v>950590</v>
       </c>
       <c r="E1983" t="inlineStr"/>
       <c r="F1983" t="inlineStr">
@@ -36209,10 +36165,8 @@
           <t>Costume de clown luxe femme M WITHOUT BRAND</t>
         </is>
       </c>
-      <c r="D1984" t="inlineStr">
-        <is>
-          <t>950590</t>
-        </is>
+      <c r="D1984" t="n">
+        <v>950590</v>
       </c>
       <c r="E1984" t="inlineStr"/>
       <c r="F1984" t="inlineStr">
@@ -36229,10 +36183,8 @@
           <t>Costume dompteur homme L WITHOUT BRAND</t>
         </is>
       </c>
-      <c r="D1985" t="inlineStr">
-        <is>
-          <t>950590</t>
-        </is>
+      <c r="D1985" t="n">
+        <v>950590</v>
       </c>
       <c r="E1985" t="inlineStr"/>
       <c r="F1985" t="inlineStr">
@@ -36249,10 +36201,8 @@
           <t>Costume dompteuse cirque rouge femme Lme WITHOUT BRAND</t>
         </is>
       </c>
-      <c r="D1986" t="inlineStr">
-        <is>
-          <t>950590</t>
-        </is>
+      <c r="D1986" t="n">
+        <v>950590</v>
       </c>
       <c r="E1986" t="inlineStr"/>
       <c r="F1986" t="inlineStr">
@@ -36269,10 +36219,8 @@
           <t>Costume dompteuse M WITHOUT BRAND</t>
         </is>
       </c>
-      <c r="D1987" t="inlineStr">
-        <is>
-          <t>950590</t>
-        </is>
+      <c r="D1987" t="n">
+        <v>950590</v>
       </c>
       <c r="E1987" t="inlineStr"/>
       <c r="F1987" t="inlineStr">
@@ -36289,10 +36237,8 @@
           <t>Costume dompteuse sexy XL WITHOUT BRAND</t>
         </is>
       </c>
-      <c r="D1988" t="inlineStr">
-        <is>
-          <t>950590</t>
-        </is>
+      <c r="D1988" t="n">
+        <v>950590</v>
       </c>
       <c r="E1988" t="inlineStr"/>
       <c r="F1988" t="inlineStr">
@@ -36309,10 +36255,8 @@
           <t>Costume dresseuse femme M WITHOUT BRAND</t>
         </is>
       </c>
-      <c r="D1989" t="inlineStr">
-        <is>
-          <t>950590</t>
-        </is>
+      <c r="D1989" t="n">
+        <v>950590</v>
       </c>
       <c r="E1989" t="inlineStr"/>
       <c r="F1989" t="inlineStr">
@@ -36329,10 +36273,8 @@
           <t>Costume femme charleston tatouée M WITHOUT BRAND</t>
         </is>
       </c>
-      <c r="D1990" t="inlineStr">
-        <is>
-          <t>950590</t>
-        </is>
+      <c r="D1990" t="n">
+        <v>950590</v>
       </c>
       <c r="E1990" t="inlineStr"/>
       <c r="F1990" t="inlineStr">
@@ -36349,10 +36291,8 @@
           <t>Costume homme fort M/L WITHOUT BRAND</t>
         </is>
       </c>
-      <c r="D1991" t="inlineStr">
-        <is>
-          <t>950590</t>
-        </is>
+      <c r="D1991" t="n">
+        <v>950590</v>
       </c>
       <c r="E1991" t="inlineStr"/>
       <c r="F1991" t="inlineStr">
@@ -36369,10 +36309,8 @@
           <t>Costume jester harley homme M/L WITHOUT BRAND</t>
         </is>
       </c>
-      <c r="D1992" t="inlineStr">
-        <is>
-          <t>950590</t>
-        </is>
+      <c r="D1992" t="n">
+        <v>950590</v>
       </c>
       <c r="E1992" t="inlineStr"/>
       <c r="F1992" t="inlineStr">
@@ -36389,10 +36327,8 @@
           <t>Veste homme sequin silver L WITHOUT BRAND</t>
         </is>
       </c>
-      <c r="D1993" t="inlineStr">
-        <is>
-          <t>950590</t>
-        </is>
+      <c r="D1993" t="n">
+        <v>950590</v>
       </c>
       <c r="E1993" t="inlineStr"/>
       <c r="F1993" t="inlineStr">
@@ -36409,10 +36345,8 @@
           <t>Veste noire époque à Galon M homme WITHOUT BRAND</t>
         </is>
       </c>
-      <c r="D1994" t="inlineStr">
-        <is>
-          <t>950590</t>
-        </is>
+      <c r="D1994" t="n">
+        <v>950590</v>
       </c>
       <c r="E1994" t="inlineStr"/>
       <c r="F1994" t="inlineStr">
@@ -36429,10 +36363,8 @@
           <t>BATONNETS BOITE DE 100</t>
         </is>
       </c>
-      <c r="D1995" t="inlineStr">
-        <is>
-          <t>442199</t>
-        </is>
+      <c r="D1995" t="n">
+        <v>442199</v>
       </c>
       <c r="E1995" t="inlineStr"/>
       <c r="F1995" t="inlineStr">
@@ -36449,10 +36381,8 @@
           <t>MARQUEURS ACRYLIQUE DIFFERENTS COLORIS BOITE DE 10</t>
         </is>
       </c>
-      <c r="D1996" t="inlineStr">
-        <is>
-          <t>960820</t>
-        </is>
+      <c r="D1996" t="n">
+        <v>960820</v>
       </c>
       <c r="E1996" t="inlineStr"/>
       <c r="F1996" t="inlineStr">
@@ -36469,10 +36399,8 @@
           <t>MINI ENCREUR POUR TAMPON DIFFERENTS COLORIS LOT DE 12</t>
         </is>
       </c>
-      <c r="D1997" t="inlineStr">
-        <is>
-          <t>961220</t>
-        </is>
+      <c r="D1997" t="n">
+        <v>961220</v>
       </c>
       <c r="E1997" t="inlineStr"/>
       <c r="F1997" t="inlineStr">
@@ -36489,10 +36417,8 @@
           <t>TAMPON ALPHABET EN MOUSSE LOT DE 42</t>
         </is>
       </c>
-      <c r="D1998" t="inlineStr">
-        <is>
-          <t>961220</t>
-        </is>
+      <c r="D1998" t="n">
+        <v>961220</v>
       </c>
       <c r="E1998" t="inlineStr"/>
       <c r="F1998" t="inlineStr">
@@ -36509,10 +36435,8 @@
           <t>TUNNEL DE MOTRICITE SEMI-TRANSPARENT LG 150 CM D.50 CM</t>
         </is>
       </c>
-      <c r="D1999" t="inlineStr">
-        <is>
-          <t>950699</t>
-        </is>
+      <c r="D1999" t="n">
+        <v>950699</v>
       </c>
       <c r="E1999" t="inlineStr"/>
       <c r="F1999" t="inlineStr">

</xml_diff>

<commit_message>
feat: add clubmed BDD xlsx
</commit_message>
<xml_diff>
--- a/data/processed/clubmed_bdd.xlsx
+++ b/data/processed/clubmed_bdd.xlsx
@@ -36448,4 +36448,365 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101007F02DC4410AE5542B5AB8CD1BCE3EB1B" ma:contentTypeVersion="18" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="33ab3980862d308bb9496ba1df291ad8">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="cd408c42-660c-44d9-b4f9-0e1628407853" xmlns:ns3="70d61308-5416-411c-9745-baf63b14e69d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="aef01502487b94b46343aea5a70672f6" ns2:_="" ns3:_="">
+    <xsd:import namespace="cd408c42-660c-44d9-b4f9-0e1628407853"/>
+    <xsd:import namespace="70d61308-5416-411c-9745-baf63b14e69d"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:_dlc_DocIdUrl" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns3:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns2:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns2:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:_dlc_DocId" minOccurs="0"/>
+                <xsd:element ref="ns2:_dlc_DocIdPersistId" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceBillingMetadata" minOccurs="0"/>
+                <xsd:element ref="ns3:NbLignes_x002e_" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="cd408c42-660c-44d9-b4f9-0e1628407853" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="_dlc_DocIdUrl" ma:index="1" nillable="true" ma:displayName="ID de document" ma:description="Lien permanent vers ce document." ma:hidden="true" ma:internalName="_dlc_DocIdUrl" ma:readOnly="false">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:URL">
+            <xsd:sequence>
+              <xsd:element name="Url" type="dms:ValidUrl" minOccurs="0" nillable="true"/>
+              <xsd:element name="Description" type="xsd:string" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="TaxCatchAll" ma:index="13" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{1e17d1a7-64de-4645-92ca-b71a87f5e83a}" ma:internalName="TaxCatchAll" ma:readOnly="false" ma:showField="CatchAllData" ma:web="cd408c42-660c-44d9-b4f9-0e1628407853">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="17" nillable="true" ma:displayName="Partagé avec" ma:hidden="true" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="18" nillable="true" ma:displayName="Partagé avec détails" ma:hidden="true" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="_dlc_DocId" ma:index="22" nillable="true" ma:displayName="Valeur d’ID de document" ma:description="Valeur de l’ID de document affecté à cet élément." ma:hidden="true" ma:indexed="true" ma:internalName="_dlc_DocId" ma:readOnly="false">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="_dlc_DocIdPersistId" ma:index="24" nillable="true" ma:displayName="Conserver l’ID" ma:description="Conserver l’ID lors de l’ajout." ma:hidden="true" ma:internalName="_dlc_DocIdPersistId" ma:readOnly="false">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Boolean"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="70d61308-5416-411c-9745-baf63b14e69d" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="10" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="12" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Balises d’images" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="3fc804f8-5688-4369-a638-782d369e9079" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="14" nillable="true" ma:displayName="Extracted Text" ma:hidden="true" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="19" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="20" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="21" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="25" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="26" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="NbLignes_x002e_" ma:index="27" nillable="true" ma:displayName="NbLignes." ma:format="Dropdown" ma:internalName="NbLignes_x002e_" ma:percentage="FALSE">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Number"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:displayName="Type de contenu"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="3" ma:displayName="Titre"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_dlc_DocId xmlns="cd408c42-660c-44d9-b4f9-0e1628407853">7HDWNRJCXEKA-370941378-286387</_dlc_DocId>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="70d61308-5416-411c-9745-baf63b14e69d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="cd408c42-660c-44d9-b4f9-0e1628407853" xsi:nil="true"/>
+    <_dlc_DocIdPersistId xmlns="cd408c42-660c-44d9-b4f9-0e1628407853" xsi:nil="true"/>
+    <_dlc_DocIdUrl xmlns="cd408c42-660c-44d9-b4f9-0e1628407853">
+      <Url>https://clubmedoffice.sharepoint.com/sites/SC-MthodesLogistiques-EAF/_layouts/15/DocIdRedir.aspx?ID=7HDWNRJCXEKA-370941378-286387</Url>
+      <Description>7HDWNRJCXEKA-370941378-286387</Description>
+    </_dlc_DocIdUrl>
+    <NbLignes_x002e_ xmlns="70d61308-5416-411c-9745-baf63b14e69d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B371A0B8-2D2F-4EB1-BA3D-20FCEA61FBB3}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7747FE9C-61E1-4D77-9BFB-EBA168D8F737}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8C43EF38-FD90-40B8-BF87-45476AA2B133}"/>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{447C9CE4-376B-4019-8E21-A7F654C8DC83}"/>
 </file>
</xml_diff>